<commit_message>
release: prepare literature-table-organizer v2
</commit_message>
<xml_diff>
--- a/assets/demo/literature-demo.xlsx
+++ b/assets/demo/literature-demo.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,6 +547,35 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Large Language Models for Orchestrating Bimanual Robots (LABOR)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2404.02018</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>An LLM-based orchestration paper for long-horizon bimanual manipulation that is useful for testing webpage fallback behavior.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add survey-oriented review workflow mode
</commit_message>
<xml_diff>
--- a/assets/demo/literature-demo.xlsx
+++ b/assets/demo/literature-demo.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,15 +480,25 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>写作引用章节</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>引用论据</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>本地文件路径</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>证据链路径</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>核验警告/状态</t>
         </is>
@@ -522,6 +532,8 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -547,6 +559,8 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -576,6 +590,8 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -588,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -761,6 +777,40 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>写作引用章节</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>指向写作大纲中的章节或子章节</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>例如 3.2 Taxonomy / 4.1 Representative methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>引用论据</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>写入可直接服务写作的具体论据</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>包含具体方法差异、数字结果或边界说明</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>